<commit_message>
Update Aze phylogeny processing
</commit_message>
<xml_diff>
--- a/1-Data_raw/Aze_phylogeny/IF_Match_fossils_and_lineages.xlsx
+++ b/1-Data_raw/Aze_phylogeny/IF_Match_fossils_and_lineages.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10520"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Jeremy/Documents/Scolaire/Stage_ESaupe/Forams/Data_processing/Processed_data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Jeremy/Nextcloud/Recherche/2_Plankton/Forams/1-Data_raw/Aze_phylogeny/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8093241C-5815-0C4D-8B43-481D16CDEEA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CC575A3-CBBD-0148-A1D7-B2ECA0A5E294}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" activeTab="1" xr2:uid="{E84BCE5F-B634-4635-8845-23AC4F181B2D}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="28800" windowHeight="17560" xr2:uid="{E84BCE5F-B634-4635-8845-23AC4F181B2D}"/>
   </bookViews>
   <sheets>
     <sheet name="Not in tree" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="304" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="164">
   <si>
     <t>Alicantina lozanoi</t>
   </si>
@@ -476,6 +476,48 @@
   </si>
   <si>
     <t>Previously indicated as Catapsydrax unicavus, but incoherent with tree topology</t>
+  </si>
+  <si>
+    <t>Fossil names (old, wrong order)</t>
+  </si>
+  <si>
+    <t>Alicantina prolata-Alicantina lozanoi</t>
+  </si>
+  <si>
+    <t>Ciperoella fariasi-Ciperoella ciperoensis</t>
+  </si>
+  <si>
+    <t>Globigerinella obesa-Globigerinella clavaticamerata</t>
+  </si>
+  <si>
+    <t>Globigerinoides ruber-Globigerinoides elongatus</t>
+  </si>
+  <si>
+    <t>Globoconella inflata-Globoconella triangula</t>
+  </si>
+  <si>
+    <t>Catapsydrax unicavus-Globorotaloides suteri</t>
+  </si>
+  <si>
+    <t>Globigerina praebulloides-Globoturborotalita occlusa</t>
+  </si>
+  <si>
+    <t>Neogloboquadrina humerosa-Neogloboquadrina atlantica</t>
+  </si>
+  <si>
+    <t>Neogloboquadrina pachyderma-Neogloboquadrina incompta</t>
+  </si>
+  <si>
+    <t>Paragloborotalia nana-Paragloborotalia pseudocontinuosa</t>
+  </si>
+  <si>
+    <t>Subbotina angiporoides-Subbotina minima</t>
+  </si>
+  <si>
+    <t>Trilobatus trilobus-Trilobatus quadrilobatus-Trilobatus praeimmaturus-Trilobatus immaturus</t>
+  </si>
+  <si>
+    <t>Trilobatus subsacculifer-Trilobatus sacculifer</t>
   </si>
 </sst>
 </file>
@@ -578,9 +620,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office 2013 – 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -618,7 +660,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -724,7 +766,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -866,7 +908,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -874,17 +916,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF38C2F2-8BED-42FE-BF55-1FA8CD2807F1}">
-  <dimension ref="A1:E48"/>
+  <dimension ref="A1:F48"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="33.5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="33.5" customWidth="1"/>
     <col min="3" max="3" width="37.1640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="73.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="28.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="88" customWidth="1"/>
+    <col min="5" max="5" width="73.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="28.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>47</v>
       </c>
@@ -895,13 +938,16 @@
         <v>107</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -912,10 +958,13 @@
         <v>136</v>
       </c>
       <c r="E2" t="s">
+        <v>151</v>
+      </c>
+      <c r="F2" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -926,10 +975,13 @@
         <v>136</v>
       </c>
       <c r="E3" t="s">
+        <v>151</v>
+      </c>
+      <c r="F3" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -940,11 +992,14 @@
       <c r="D4" t="s">
         <v>2</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" t="s">
+        <v>2</v>
+      </c>
+      <c r="F4" s="3" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -955,11 +1010,14 @@
       <c r="D5" t="s">
         <v>3</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" t="s">
+        <v>3</v>
+      </c>
+      <c r="F5" s="3" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -970,11 +1028,14 @@
       <c r="D6" t="s">
         <v>137</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="E6" t="s">
+        <v>152</v>
+      </c>
+      <c r="F6" s="3" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -984,11 +1045,14 @@
       <c r="D7" t="s">
         <v>137</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="E7" t="s">
+        <v>152</v>
+      </c>
+      <c r="F7" s="3" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>6</v>
       </c>
@@ -998,8 +1062,11 @@
       <c r="D8" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="E8" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>7</v>
       </c>
@@ -1010,11 +1077,14 @@
       <c r="D9" t="s">
         <v>7</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="E9" t="s">
+        <v>7</v>
+      </c>
+      <c r="F9" s="3" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -1025,11 +1095,14 @@
       <c r="D10" t="s">
         <v>8</v>
       </c>
-      <c r="E10" s="3" t="s">
+      <c r="E10" t="s">
+        <v>8</v>
+      </c>
+      <c r="F10" s="3" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -1040,10 +1113,13 @@
         <v>138</v>
       </c>
       <c r="E11" t="s">
+        <v>153</v>
+      </c>
+      <c r="F11" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>10</v>
       </c>
@@ -1053,8 +1129,11 @@
       <c r="D12" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="E12" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>11</v>
       </c>
@@ -1065,11 +1144,14 @@
       <c r="D13" t="s">
         <v>11</v>
       </c>
-      <c r="E13" s="3" t="s">
+      <c r="E13" t="s">
+        <v>11</v>
+      </c>
+      <c r="F13" s="3" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>12</v>
       </c>
@@ -1080,11 +1162,14 @@
       <c r="D14" t="s">
         <v>12</v>
       </c>
-      <c r="E14" s="3" t="s">
+      <c r="E14" t="s">
+        <v>12</v>
+      </c>
+      <c r="F14" s="3" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>13</v>
       </c>
@@ -1095,10 +1180,13 @@
         <v>139</v>
       </c>
       <c r="E15" t="s">
+        <v>154</v>
+      </c>
+      <c r="F15" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>14</v>
       </c>
@@ -1109,11 +1197,14 @@
       <c r="D16" t="s">
         <v>14</v>
       </c>
-      <c r="E16" s="3" t="s">
+      <c r="E16" t="s">
+        <v>14</v>
+      </c>
+      <c r="F16" s="3" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>15</v>
       </c>
@@ -1124,11 +1215,14 @@
       <c r="D17" t="s">
         <v>15</v>
       </c>
-      <c r="E17" s="3" t="s">
+      <c r="E17" t="s">
+        <v>15</v>
+      </c>
+      <c r="F17" s="3" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>16</v>
       </c>
@@ -1139,10 +1233,13 @@
         <v>16</v>
       </c>
       <c r="E18" t="s">
+        <v>16</v>
+      </c>
+      <c r="F18" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>17</v>
       </c>
@@ -1153,10 +1250,13 @@
         <v>140</v>
       </c>
       <c r="E19" t="s">
+        <v>155</v>
+      </c>
+      <c r="F19" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>18</v>
       </c>
@@ -1167,11 +1267,14 @@
       <c r="D20" t="s">
         <v>18</v>
       </c>
-      <c r="E20" s="3" t="s">
+      <c r="E20" t="s">
+        <v>18</v>
+      </c>
+      <c r="F20" s="3" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>19</v>
       </c>
@@ -1182,11 +1285,14 @@
       <c r="D21" t="s">
         <v>19</v>
       </c>
-      <c r="E21" s="3" t="s">
+      <c r="E21" t="s">
+        <v>19</v>
+      </c>
+      <c r="F21" s="3" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>20</v>
       </c>
@@ -1197,10 +1303,13 @@
         <v>141</v>
       </c>
       <c r="E22" t="s">
+        <v>156</v>
+      </c>
+      <c r="F22" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>21</v>
       </c>
@@ -1210,11 +1319,14 @@
       <c r="D23" t="s">
         <v>21</v>
       </c>
-      <c r="E23" s="3" t="s">
+      <c r="E23" t="s">
+        <v>21</v>
+      </c>
+      <c r="F23" s="3" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>22</v>
       </c>
@@ -1224,8 +1336,11 @@
       <c r="D24" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="E24" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>23</v>
       </c>
@@ -1236,11 +1351,14 @@
       <c r="D25" t="s">
         <v>23</v>
       </c>
-      <c r="E25" s="3" t="s">
+      <c r="E25" t="s">
+        <v>23</v>
+      </c>
+      <c r="F25" s="3" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>24</v>
       </c>
@@ -1251,11 +1369,14 @@
       <c r="D26" t="s">
         <v>24</v>
       </c>
-      <c r="E26" s="3" t="s">
+      <c r="E26" t="s">
+        <v>24</v>
+      </c>
+      <c r="F26" s="3" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>25</v>
       </c>
@@ -1266,10 +1387,13 @@
         <v>142</v>
       </c>
       <c r="E27" t="s">
+        <v>157</v>
+      </c>
+      <c r="F27" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>26</v>
       </c>
@@ -1280,11 +1404,14 @@
       <c r="D28" t="s">
         <v>26</v>
       </c>
-      <c r="E28" s="3" t="s">
+      <c r="E28" t="s">
+        <v>26</v>
+      </c>
+      <c r="F28" s="3" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>27</v>
       </c>
@@ -1295,11 +1422,14 @@
       <c r="D29" t="s">
         <v>27</v>
       </c>
-      <c r="E29" s="3" t="s">
+      <c r="E29" t="s">
+        <v>27</v>
+      </c>
+      <c r="F29" s="3" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>28</v>
       </c>
@@ -1310,11 +1440,14 @@
       <c r="D30" t="s">
         <v>28</v>
       </c>
-      <c r="E30" s="3" t="s">
+      <c r="E30" t="s">
+        <v>28</v>
+      </c>
+      <c r="F30" s="3" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>29</v>
       </c>
@@ -1325,10 +1458,13 @@
         <v>143</v>
       </c>
       <c r="E31" t="s">
+        <v>158</v>
+      </c>
+      <c r="F31" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>30</v>
       </c>
@@ -1339,10 +1475,13 @@
         <v>145</v>
       </c>
       <c r="E32" t="s">
+        <v>159</v>
+      </c>
+      <c r="F32" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>31</v>
       </c>
@@ -1353,11 +1492,14 @@
       <c r="D33" t="s">
         <v>31</v>
       </c>
-      <c r="E33" s="3" t="s">
+      <c r="E33" t="s">
+        <v>31</v>
+      </c>
+      <c r="F33" s="3" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>32</v>
       </c>
@@ -1368,11 +1510,14 @@
       <c r="D34" t="s">
         <v>32</v>
       </c>
-      <c r="E34" s="3" t="s">
+      <c r="E34" t="s">
+        <v>32</v>
+      </c>
+      <c r="F34" s="3" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>33</v>
       </c>
@@ -1383,10 +1528,13 @@
         <v>144</v>
       </c>
       <c r="E35" t="s">
+        <v>160</v>
+      </c>
+      <c r="F35" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>34</v>
       </c>
@@ -1397,11 +1545,14 @@
       <c r="D36" t="s">
         <v>34</v>
       </c>
-      <c r="E36" s="3" t="s">
+      <c r="E36" t="s">
+        <v>34</v>
+      </c>
+      <c r="F36" s="3" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>35</v>
       </c>
@@ -1412,11 +1563,14 @@
       <c r="D37" t="s">
         <v>35</v>
       </c>
-      <c r="E37" s="3" t="s">
+      <c r="E37" t="s">
+        <v>35</v>
+      </c>
+      <c r="F37" s="3" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>36</v>
       </c>
@@ -1427,11 +1581,14 @@
       <c r="D38" t="s">
         <v>36</v>
       </c>
-      <c r="E38" s="3" t="s">
+      <c r="E38" t="s">
+        <v>36</v>
+      </c>
+      <c r="F38" s="3" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>37</v>
       </c>
@@ -1442,10 +1599,13 @@
         <v>146</v>
       </c>
       <c r="E39" t="s">
+        <v>161</v>
+      </c>
+      <c r="F39" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>38</v>
       </c>
@@ -1456,11 +1616,14 @@
       <c r="D40" t="s">
         <v>38</v>
       </c>
-      <c r="E40" s="3" t="s">
+      <c r="E40" t="s">
+        <v>38</v>
+      </c>
+      <c r="F40" s="3" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>39</v>
       </c>
@@ -1470,11 +1633,14 @@
       <c r="D41" t="s">
         <v>147</v>
       </c>
-      <c r="E41" s="3" t="s">
+      <c r="E41" t="s">
+        <v>162</v>
+      </c>
+      <c r="F41" s="3" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>40</v>
       </c>
@@ -1484,11 +1650,14 @@
       <c r="D42" t="s">
         <v>147</v>
       </c>
-      <c r="E42" s="3" t="s">
+      <c r="E42" t="s">
+        <v>162</v>
+      </c>
+      <c r="F42" s="3" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>41</v>
       </c>
@@ -1499,11 +1668,14 @@
       <c r="D43" t="s">
         <v>41</v>
       </c>
-      <c r="E43" s="3" t="s">
+      <c r="E43" t="s">
+        <v>41</v>
+      </c>
+      <c r="F43" s="3" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>42</v>
       </c>
@@ -1513,11 +1685,14 @@
       <c r="D44" t="s">
         <v>147</v>
       </c>
-      <c r="E44" s="3" t="s">
+      <c r="E44" t="s">
+        <v>162</v>
+      </c>
+      <c r="F44" s="3" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>43</v>
       </c>
@@ -1528,11 +1703,14 @@
       <c r="D45" t="s">
         <v>148</v>
       </c>
-      <c r="E45" s="3" t="s">
+      <c r="E45" t="s">
+        <v>163</v>
+      </c>
+      <c r="F45" s="3" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>44</v>
       </c>
@@ -1543,11 +1721,14 @@
       <c r="D46" t="s">
         <v>44</v>
       </c>
-      <c r="E46" s="3" t="s">
+      <c r="E46" t="s">
+        <v>44</v>
+      </c>
+      <c r="F46" s="3" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>45</v>
       </c>
@@ -1557,11 +1738,14 @@
       <c r="D47" t="s">
         <v>148</v>
       </c>
-      <c r="E47" s="3" t="s">
+      <c r="E47" t="s">
+        <v>163</v>
+      </c>
+      <c r="F47" s="3" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>46</v>
       </c>
@@ -1572,7 +1756,10 @@
       <c r="D48" t="s">
         <v>147</v>
       </c>
-      <c r="E48" s="3" t="s">
+      <c r="E48" t="s">
+        <v>162</v>
+      </c>
+      <c r="F48" s="3" t="s">
         <v>67</v>
       </c>
     </row>

</xml_diff>